<commit_message>
fix: strip author, threaded comments and tenant label from the register template
Removes xl/persons, xl/threadedComments, the legacy comments and VML shapes they mirror, and docMetadata/LabelInfo.xml, plus their relationships, content types and the sheet's legacyDrawing. Sheet, styles and shared strings are unchanged.
</commit_message>
<xml_diff>
--- a/frontend/public/analysis-register-template.xlsx
+++ b/frontend/public/analysis-register-template.xlsx
@@ -11,33 +11,6 @@
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={D38D9C52-0E82-4EB3-8B74-95FEE4C16B48}</author>
-    <author>tc={6A5ADE87-9C5E-4441-B725-059F80B6DB89}</author>
-  </authors>
-  <commentList>
-    <comment ref="E26" authorId="0" shapeId="0" xr:uid="{D38D9C52-0E82-4EB3-8B74-95FEE4C16B48}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Conditional formatting this column if cell says “Y”</t>
-      </text>
-    </comment>
-    <comment ref="F26" authorId="1" shapeId="0" xr:uid="{6A5ADE87-9C5E-4441-B725-059F80B6DB89}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Conditional formatting this column if cell says “Y”</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -539,12 +512,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Mary K. Kretschmar" id="{9500082C-2F98-4A65-B93F-F5943FC9CE70}" userId="S::MKKretschmar@sgh.com::fbe27c88-8b4f-417a-9bde-332fca4bff51" providerId="AD"/>
-</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -862,17 +829,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="E26" dT="2025-11-14T17:35:45.90" personId="{9500082C-2F98-4A65-B93F-F5943FC9CE70}" id="{D38D9C52-0E82-4EB3-8B74-95FEE4C16B48}">
-    <text>Conditional formatting this column if cell says “Y”</text>
-  </threadedComment>
-  <threadedComment ref="F26" dT="2025-11-14T17:35:41.40" personId="{9500082C-2F98-4A65-B93F-F5943FC9CE70}" id="{6A5ADE87-9C5E-4441-B725-059F80B6DB89}">
-    <text>Conditional formatting this column if cell says “Y”</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{691D12D9-C02E-4CA4-BC48-17C71AFEDE6A}">
   <dimension ref="A2:H54"/>
@@ -1365,12 +1321,5 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{3ce735c3-3481-4338-97d1-a7e212711caf}" enabled="0" method="" siteId="{3ce735c3-3481-4338-97d1-a7e212711caf}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>